<commit_message>
feat(parser): integration tests and fixtures (P3-L)
</commit_message>
<xml_diff>
--- a/crates/prokuroParser/tests/fixtures/minimal.xlsx
+++ b/crates/prokuroParser/tests/fixtures/minimal.xlsx
@@ -3,49 +3,88 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
-    <sheet name="Notes" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>mpn</t>
+          <t>MPN</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Manufacturer</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>qty</t>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>RefDes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RC0603FR-0710KL</t>
+          <t>GRM155R61A104KA01D</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Murata</t>
         </is>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Capacitor 100nF 10V X5R 0402</t>
+        </is>
       </c>
     </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>CRCW060310K0FKEA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Vishay</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>R1;R2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Resistor 10k 1% 0603</t>
         </is>
       </c>
     </row>

</xml_diff>